<commit_message>
Client And JLCPCB BOM Updated
Matrix Board.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Client_BOM_John_Main.xlsx
+++ b/Deliverables/BOM/Client_BOM_John_Main.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\JohnWollam-MatrixProject\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="242">
   <si>
     <t>#</t>
   </si>
@@ -742,13 +742,16 @@
   </si>
   <si>
     <t>STMicroelectronics</t>
+  </si>
+  <si>
+    <t>DO NOT MOUNT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -787,6 +790,14 @@
     <font>
       <b/>
       <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -907,7 +918,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -946,6 +957,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1871,7 +1891,7 @@
       </c>
       <c r="K20" s="9"/>
     </row>
-    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
@@ -1880,26 +1900,30 @@
       <c r="C21" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="15" t="s">
         <v>232</v>
       </c>
-      <c r="G21" s="8" t="s">
+      <c r="G21" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="H21" s="7"/>
-      <c r="I21" s="10" t="s">
+      <c r="H21" s="15" t="s">
         <v>239</v>
       </c>
-      <c r="J21" s="7">
+      <c r="I21" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="J21" s="15">
         <v>7</v>
       </c>
-      <c r="K21" s="7"/>
+      <c r="K21" s="15" t="s">
+        <v>241</v>
+      </c>
     </row>
     <row r="22" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>

</xml_diff>